<commit_message>
Update test files and CI tools
</commit_message>
<xml_diff>
--- a/src/test/resources/LoginData/LoginData.xlsx
+++ b/src/test/resources/LoginData/LoginData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30516"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ACE2B31F-0ECB-4457-A263-A638C4162863}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FDFCC9DB-D73C-4845-BD71-9969AB139A36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
     <t>Valid login</t>
   </si>
   <si>
-    <t>user_t5g34v@shopease.com</t>
+    <t>user_t5g34v@shopeae.com</t>
   </si>
   <si>
     <t>Test@3718</t>
@@ -577,7 +577,7 @@
       <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D2" t="s">
@@ -808,6 +808,7 @@
     <hyperlink ref="C13" r:id="rId8" xr:uid="{23FC19B9-643A-446F-81D0-07AE3AE9D28E}"/>
     <hyperlink ref="C14" r:id="rId9" xr:uid="{28D423A7-877E-4B30-99BD-63CE732102E2}"/>
     <hyperlink ref="C15" r:id="rId10" xr:uid="{61A5DC07-0720-492D-8588-A52D0B992567}"/>
+    <hyperlink ref="C2" r:id="rId11" xr:uid="{3F531B3E-7EA1-4EBE-97BE-8C1D6BB81F9D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>